<commit_message>
Update X5 KK Perempuan Bekerja 2024.xlsx
</commit_message>
<xml_diff>
--- a/Data terbaru dip/X5 Persentase kepala keluarga perempuan yang bekerja/2024/X5 KK Perempuan Bekerja 2024.xlsx
+++ b/Data terbaru dip/X5 Persentase kepala keluarga perempuan yang bekerja/2024/X5 KK Perempuan Bekerja 2024.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\1. File Kuliah\3. Lomba\satria data\Dataa off\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\1. File Kuliah\3. Lomba\satria data\womanguard-index-surabaya\Data terbaru dip\X5 Persentase kepala keluarga perempuan yang bekerja\2024\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0775CD58-BA90-411C-9ABB-B3D86775B738}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E97E4AB-752D-49EE-85E4-C368C4EA965D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{05CB65E3-FFAD-4C76-B546-07361076235E}"/>
   </bookViews>
@@ -1156,7 +1156,7 @@
     <col min="92" max="92" width="17.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:181" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:181" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1181,523 +1181,523 @@
       <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="Z1" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AA1" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="AB1" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="AC1" t="s">
+      <c r="AC1" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="AD1" t="s">
+      <c r="AD1" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="AE1" t="s">
+      <c r="AE1" s="6" t="s">
         <v>94</v>
       </c>
-      <c r="AF1" t="s">
+      <c r="AF1" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="AG1" t="s">
+      <c r="AG1" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="AH1" t="s">
+      <c r="AH1" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="AI1" t="s">
+      <c r="AI1" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="AJ1" t="s">
+      <c r="AJ1" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="AK1" t="s">
+      <c r="AK1" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="AL1" t="s">
+      <c r="AL1" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="AM1" t="s">
+      <c r="AM1" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="AN1" t="s">
+      <c r="AN1" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="AO1" t="s">
+      <c r="AO1" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="AP1" t="s">
+      <c r="AP1" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="AQ1" t="s">
+      <c r="AQ1" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="AR1" t="s">
+      <c r="AR1" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="AS1" t="s">
+      <c r="AS1" s="6" t="s">
         <v>108</v>
       </c>
-      <c r="AT1" t="s">
+      <c r="AT1" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="AU1" t="s">
+      <c r="AU1" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="AV1" t="s">
+      <c r="AV1" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="AW1" t="s">
+      <c r="AW1" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="AX1" t="s">
+      <c r="AX1" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="AY1" t="s">
+      <c r="AY1" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="AZ1" t="s">
+      <c r="AZ1" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="BA1" t="s">
+      <c r="BA1" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="BB1" t="s">
+      <c r="BB1" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="BC1" t="s">
+      <c r="BC1" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="BD1" t="s">
+      <c r="BD1" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="BE1" t="s">
+      <c r="BE1" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="BF1" t="s">
+      <c r="BF1" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="BG1" t="s">
+      <c r="BG1" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="BH1" t="s">
+      <c r="BH1" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="BI1" t="s">
+      <c r="BI1" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="BJ1" t="s">
+      <c r="BJ1" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="BK1" t="s">
+      <c r="BK1" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="BL1" t="s">
+      <c r="BL1" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="BM1" t="s">
+      <c r="BM1" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="BN1" t="s">
+      <c r="BN1" s="6" t="s">
         <v>129</v>
       </c>
-      <c r="BO1" t="s">
+      <c r="BO1" s="6" t="s">
         <v>130</v>
       </c>
-      <c r="BP1" t="s">
+      <c r="BP1" s="6" t="s">
         <v>131</v>
       </c>
-      <c r="BQ1" t="s">
+      <c r="BQ1" s="6" t="s">
         <v>132</v>
       </c>
-      <c r="BR1" t="s">
+      <c r="BR1" s="6" t="s">
         <v>133</v>
       </c>
-      <c r="BS1" t="s">
+      <c r="BS1" s="6" t="s">
         <v>134</v>
       </c>
-      <c r="BT1" t="s">
+      <c r="BT1" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="BU1" t="s">
+      <c r="BU1" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="BV1" t="s">
+      <c r="BV1" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="BW1" t="s">
+      <c r="BW1" s="6" t="s">
         <v>138</v>
       </c>
-      <c r="BX1" t="s">
+      <c r="BX1" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="BY1" t="s">
+      <c r="BY1" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="BZ1" t="s">
+      <c r="BZ1" s="6" t="s">
         <v>141</v>
       </c>
-      <c r="CA1" t="s">
+      <c r="CA1" s="6" t="s">
         <v>142</v>
       </c>
-      <c r="CB1" t="s">
+      <c r="CB1" s="6" t="s">
         <v>143</v>
       </c>
-      <c r="CC1" t="s">
+      <c r="CC1" s="6" t="s">
         <v>144</v>
       </c>
-      <c r="CD1" t="s">
+      <c r="CD1" s="6" t="s">
         <v>145</v>
       </c>
-      <c r="CE1" t="s">
+      <c r="CE1" s="6" t="s">
         <v>146</v>
       </c>
-      <c r="CF1" t="s">
+      <c r="CF1" s="6" t="s">
         <v>147</v>
       </c>
-      <c r="CG1" t="s">
+      <c r="CG1" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="CH1" t="s">
+      <c r="CH1" s="6" t="s">
         <v>149</v>
       </c>
-      <c r="CI1" t="s">
+      <c r="CI1" s="6" t="s">
         <v>150</v>
       </c>
-      <c r="CJ1" t="s">
+      <c r="CJ1" s="6" t="s">
         <v>151</v>
       </c>
-      <c r="CK1" t="s">
+      <c r="CK1" s="6" t="s">
         <v>152</v>
       </c>
-      <c r="CL1" t="s">
+      <c r="CL1" s="6" t="s">
         <v>153</v>
       </c>
-      <c r="CM1" t="s">
+      <c r="CM1" s="6" t="s">
         <v>154</v>
       </c>
-      <c r="CN1" t="s">
+      <c r="CN1" s="6" t="s">
         <v>155</v>
       </c>
-      <c r="CO1" t="s">
+      <c r="CO1" s="6" t="s">
         <v>156</v>
       </c>
-      <c r="CP1" t="s">
+      <c r="CP1" s="6" t="s">
         <v>157</v>
       </c>
-      <c r="CQ1" t="s">
+      <c r="CQ1" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="CR1" t="s">
+      <c r="CR1" s="6" t="s">
         <v>159</v>
       </c>
-      <c r="CS1" t="s">
+      <c r="CS1" s="6" t="s">
         <v>160</v>
       </c>
-      <c r="CT1" t="s">
+      <c r="CT1" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="CU1" t="s">
+      <c r="CU1" s="6" t="s">
         <v>162</v>
       </c>
-      <c r="CV1" t="s">
+      <c r="CV1" s="6" t="s">
         <v>163</v>
       </c>
-      <c r="CW1" t="s">
+      <c r="CW1" s="6" t="s">
         <v>164</v>
       </c>
-      <c r="CX1" t="s">
+      <c r="CX1" s="6" t="s">
         <v>165</v>
       </c>
-      <c r="CY1" t="s">
+      <c r="CY1" s="6" t="s">
         <v>166</v>
       </c>
-      <c r="CZ1" t="s">
+      <c r="CZ1" s="6" t="s">
         <v>167</v>
       </c>
-      <c r="DA1" t="s">
+      <c r="DA1" s="6" t="s">
         <v>168</v>
       </c>
-      <c r="DB1" t="s">
+      <c r="DB1" s="6" t="s">
         <v>169</v>
       </c>
-      <c r="DC1" t="s">
+      <c r="DC1" s="6" t="s">
         <v>170</v>
       </c>
-      <c r="DD1" t="s">
+      <c r="DD1" s="6" t="s">
         <v>171</v>
       </c>
-      <c r="DE1" t="s">
+      <c r="DE1" s="6" t="s">
         <v>172</v>
       </c>
       <c r="DF1" s="6" t="s">
         <v>173</v>
       </c>
-      <c r="DG1" t="s">
+      <c r="DG1" s="6" t="s">
         <v>174</v>
       </c>
-      <c r="DH1" t="s">
+      <c r="DH1" s="6" t="s">
         <v>175</v>
       </c>
-      <c r="DI1" t="s">
+      <c r="DI1" s="6" t="s">
         <v>176</v>
       </c>
-      <c r="DJ1" t="s">
+      <c r="DJ1" s="6" t="s">
         <v>177</v>
       </c>
-      <c r="DK1" t="s">
+      <c r="DK1" s="6" t="s">
         <v>178</v>
       </c>
-      <c r="DL1" t="s">
+      <c r="DL1" s="6" t="s">
         <v>179</v>
       </c>
-      <c r="DM1" t="s">
+      <c r="DM1" s="6" t="s">
         <v>180</v>
       </c>
-      <c r="DN1" t="s">
+      <c r="DN1" s="6" t="s">
         <v>181</v>
       </c>
-      <c r="DO1" t="s">
+      <c r="DO1" s="6" t="s">
         <v>182</v>
       </c>
-      <c r="DP1" t="s">
+      <c r="DP1" s="6" t="s">
         <v>183</v>
       </c>
-      <c r="DQ1" t="s">
+      <c r="DQ1" s="6" t="s">
         <v>184</v>
       </c>
-      <c r="DR1" t="s">
+      <c r="DR1" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="DS1" t="s">
+      <c r="DS1" s="6" t="s">
         <v>186</v>
       </c>
-      <c r="DT1" t="s">
+      <c r="DT1" s="6" t="s">
         <v>187</v>
       </c>
-      <c r="DU1" t="s">
+      <c r="DU1" s="6" t="s">
         <v>188</v>
       </c>
-      <c r="DV1" t="s">
+      <c r="DV1" s="6" t="s">
         <v>189</v>
       </c>
-      <c r="DW1" t="s">
+      <c r="DW1" s="6" t="s">
         <v>190</v>
       </c>
       <c r="DX1" s="6" t="s">
         <v>191</v>
       </c>
-      <c r="DY1" t="s">
+      <c r="DY1" s="6" t="s">
         <v>192</v>
       </c>
-      <c r="DZ1" t="s">
+      <c r="DZ1" s="6" t="s">
         <v>193</v>
       </c>
-      <c r="EA1" t="s">
+      <c r="EA1" s="6" t="s">
         <v>194</v>
       </c>
-      <c r="EB1" t="s">
+      <c r="EB1" s="6" t="s">
         <v>195</v>
       </c>
-      <c r="EC1" t="s">
+      <c r="EC1" s="6" t="s">
         <v>196</v>
       </c>
-      <c r="ED1" t="s">
+      <c r="ED1" s="6" t="s">
         <v>197</v>
       </c>
-      <c r="EE1" t="s">
+      <c r="EE1" s="6" t="s">
         <v>198</v>
       </c>
-      <c r="EF1" t="s">
+      <c r="EF1" s="6" t="s">
         <v>199</v>
       </c>
-      <c r="EG1" t="s">
+      <c r="EG1" s="6" t="s">
         <v>200</v>
       </c>
-      <c r="EH1" t="s">
+      <c r="EH1" s="6" t="s">
         <v>201</v>
       </c>
-      <c r="EI1" t="s">
+      <c r="EI1" s="6" t="s">
         <v>202</v>
       </c>
-      <c r="EJ1" t="s">
+      <c r="EJ1" s="6" t="s">
         <v>203</v>
       </c>
-      <c r="EK1" t="s">
+      <c r="EK1" s="6" t="s">
         <v>204</v>
       </c>
-      <c r="EL1" t="s">
+      <c r="EL1" s="6" t="s">
         <v>205</v>
       </c>
-      <c r="EM1" t="s">
+      <c r="EM1" s="6" t="s">
         <v>206</v>
       </c>
-      <c r="EN1" t="s">
+      <c r="EN1" s="6" t="s">
         <v>207</v>
       </c>
-      <c r="EO1" t="s">
+      <c r="EO1" s="6" t="s">
         <v>208</v>
       </c>
-      <c r="EP1" t="s">
+      <c r="EP1" s="6" t="s">
         <v>209</v>
       </c>
-      <c r="EQ1" t="s">
+      <c r="EQ1" s="6" t="s">
         <v>210</v>
       </c>
-      <c r="ER1" t="s">
+      <c r="ER1" s="6" t="s">
         <v>211</v>
       </c>
-      <c r="ES1" t="s">
+      <c r="ES1" s="6" t="s">
         <v>212</v>
       </c>
-      <c r="ET1" t="s">
+      <c r="ET1" s="6" t="s">
         <v>213</v>
       </c>
-      <c r="EU1" t="s">
+      <c r="EU1" s="6" t="s">
         <v>214</v>
       </c>
-      <c r="EV1" t="s">
+      <c r="EV1" s="6" t="s">
         <v>215</v>
       </c>
-      <c r="EW1" t="s">
+      <c r="EW1" s="6" t="s">
         <v>216</v>
       </c>
-      <c r="EX1" t="s">
+      <c r="EX1" s="6" t="s">
         <v>217</v>
       </c>
-      <c r="EY1" t="s">
+      <c r="EY1" s="6" t="s">
         <v>218</v>
       </c>
-      <c r="EZ1" t="s">
+      <c r="EZ1" s="6" t="s">
         <v>219</v>
       </c>
-      <c r="FA1" t="s">
+      <c r="FA1" s="6" t="s">
         <v>220</v>
       </c>
-      <c r="FB1" t="s">
+      <c r="FB1" s="6" t="s">
         <v>221</v>
       </c>
-      <c r="FC1" t="s">
+      <c r="FC1" s="6" t="s">
         <v>222</v>
       </c>
-      <c r="FD1" t="s">
+      <c r="FD1" s="6" t="s">
         <v>223</v>
       </c>
-      <c r="FE1" t="s">
+      <c r="FE1" s="6" t="s">
         <v>224</v>
       </c>
-      <c r="FF1" t="s">
+      <c r="FF1" s="6" t="s">
         <v>225</v>
       </c>
-      <c r="FG1" t="s">
+      <c r="FG1" s="6" t="s">
         <v>226</v>
       </c>
-      <c r="FH1" t="s">
+      <c r="FH1" s="6" t="s">
         <v>227</v>
       </c>
-      <c r="FI1" t="s">
+      <c r="FI1" s="6" t="s">
         <v>228</v>
       </c>
-      <c r="FJ1" t="s">
+      <c r="FJ1" s="6" t="s">
         <v>229</v>
       </c>
-      <c r="FK1" t="s">
+      <c r="FK1" s="6" t="s">
         <v>230</v>
       </c>
-      <c r="FL1" t="s">
+      <c r="FL1" s="6" t="s">
         <v>231</v>
       </c>
-      <c r="FM1" t="s">
+      <c r="FM1" s="6" t="s">
         <v>232</v>
       </c>
-      <c r="FN1" t="s">
+      <c r="FN1" s="6" t="s">
         <v>233</v>
       </c>
-      <c r="FO1" t="s">
+      <c r="FO1" s="6" t="s">
         <v>234</v>
       </c>
-      <c r="FP1" t="s">
+      <c r="FP1" s="6" t="s">
         <v>235</v>
       </c>
-      <c r="FQ1" t="s">
+      <c r="FQ1" s="6" t="s">
         <v>236</v>
       </c>
-      <c r="FR1" t="s">
+      <c r="FR1" s="6" t="s">
         <v>237</v>
       </c>
-      <c r="FS1" t="s">
+      <c r="FS1" s="6" t="s">
         <v>238</v>
       </c>
-      <c r="FT1" t="s">
+      <c r="FT1" s="6" t="s">
         <v>239</v>
       </c>
-      <c r="FU1" t="s">
+      <c r="FU1" s="6" t="s">
         <v>240</v>
       </c>
-      <c r="FV1" t="s">
+      <c r="FV1" s="6" t="s">
         <v>241</v>
       </c>
-      <c r="FW1" t="s">
+      <c r="FW1" s="6" t="s">
         <v>242</v>
       </c>
-      <c r="FX1" t="s">
+      <c r="FX1" s="6" t="s">
         <v>243</v>
       </c>
-      <c r="FY1" t="s">
+      <c r="FY1" s="6" t="s">
         <v>244</v>
       </c>
     </row>

</xml_diff>